<commit_message>
feat: add training evaluation and login regression
</commit_message>
<xml_diff>
--- a/test_cases/standard.xlsx
+++ b/test_cases/standard.xlsx
@@ -678,7 +678,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -697,6 +697,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1111,7 +1114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1"/>
   <sheetData>
     <row r="1">
@@ -1275,6 +1278,423 @@
         </is>
       </c>
       <c r="Q2" s="7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>账号登录</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>登录失败-未选择门店</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>4.点击登录</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>打开登录页面</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>1.输入 {{credential.username}}
+2.输入 {{credential.password}}
+3.不选择门店
+4.点击登录</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>input[type='text'] | input[type='password'] | button:has-text('登 录')</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>input | input | click</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>{{credential.username}} | {{credential.password}}</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>请选择门店</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>请选择门店</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>text_contains</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>探索模式自动生成</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>账号登录</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>查看用户协议</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2.直接点击页面最下方'《用户协议》'</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>打开登录页面</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>1.不输入账号和密码
+2.直接点击页面最下方'《用户协议》'</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>a:has-text('用户协议')</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>用户协议</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>/user-agreement</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>url_contains</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>探索模式自动生成</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-007</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>账号登录</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>登录成功</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>4.点击登录</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>打开登录页面</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>1.输入 {{credential.username}}
+2.输入 {{credential.password}}
+3.选择门店
+4.点击登录</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>input[type='text'] | input[type='password'] | .ant-select-selector | button:has-text('登 录')</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>input | input | select | click</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{{credential.username}} | {{credential.password}} | </t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>登录成功，跳转到首页</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>/login</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>url_not_contains</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>探索模式自动生成</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>账号登录</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>登录失败-账号密码为空</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2.点击登录按钮</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>打开登录页面</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>1.不输入账号和密码
+2.点击登录按钮</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>button:has-text('登 录')</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>请输入账号、请输入密码、请选择门店</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>请输入账号 | 请输入密码 | 请选择门店</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>text_contains_all</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>探索模式自动生成</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>账号登录</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>登录失败-密码为空</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>3.点击登录</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>打开登录页面</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>1.输入 {{credential.username}}
+2.不输入密码
+3.点击登录</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>input[type='text'] | button:has-text('登 录')</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>input | click</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>{{credential.username}}</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>请输入密码、请选择门店</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>请输入密码 | 请选择门店</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>text_contains_all</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>探索模式自动生成</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
         <is>
           <t>pass</t>
         </is>

</xml_diff>